<commit_message>
Obras con varias líneas, reparaciones, registro de soldadores y fotos por junta (v16)
- Obras y líneas: cada isométrico se guarda solo en el equipo (IndexedDB);
  abrir, nueva línea, duplicar, borrar, exportar/importar obra completa
- Reparaciones W5-R1, W5-R2…: registro propio, salen en el QC-F-004 y en
  el reporte de avance como evento REPARACION (tarifa propia en el maestro)
- Registro de soldadores (estampa, procesos, Ø mín/máx, WPQ, vencimiento)
  con avisos al asignar y % de rechazo por soldador; estampa en reportes
- Fotos por junta desde la cámara o galería (reducidas) y anexo fotográfico
- Reporte semanal de toda la obra con avance por línea

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014GD4R4MUda5s9mdoi9LkUR
</commit_message>
<xml_diff>
--- a/isometrico/plantillas/Maestro_Gerencia_Avance.xlsx
+++ b/isometrico/plantillas/Maestro_Gerencia_Avance.xlsx
@@ -485,7 +485,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -606,6 +606,13 @@
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>TALLER = soldadura en taller (S, shop weld). CAMPO = soldadura en campo (F, field weld). SIN DEFINIR = la junta no tiene taller/campo: corríjalo en la obra.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>REPARACIÓN = soldadura de reparación de una junta rechazada (W5-R1, W5-R2…). Póngale tarifa positiva para cobrarla o negativa para descontarla.</t>
         </is>
       </c>
     </row>
@@ -620,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -628,6 +635,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -656,6 +664,11 @@
           <t>CAMPO LIBERADO $/ML</t>
         </is>
       </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>REPARACIÓN $/ML (negativo = descuento)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -675,6 +688,9 @@
       <c r="E2" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F2" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -694,6 +710,9 @@
       <c r="E3" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F3" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -713,6 +732,9 @@
       <c r="E4" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F4" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -732,6 +754,9 @@
       <c r="E5" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F5" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -751,6 +776,9 @@
       <c r="E6" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F6" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -770,6 +798,9 @@
       <c r="E7" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F7" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -789,6 +820,9 @@
       <c r="E8" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -808,6 +842,9 @@
       <c r="E9" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F9" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -827,6 +864,9 @@
       <c r="E10" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -846,6 +886,9 @@
       <c r="E11" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F11" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -865,6 +908,9 @@
       <c r="E12" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -884,6 +930,9 @@
       <c r="E13" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F13" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -903,6 +952,9 @@
       <c r="E14" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -922,6 +974,9 @@
       <c r="E15" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F15" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -941,6 +996,9 @@
       <c r="E16" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -960,6 +1018,9 @@
       <c r="E17" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -979,6 +1040,9 @@
       <c r="E18" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -998,6 +1062,9 @@
       <c r="E19" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1017,6 +1084,9 @@
       <c r="E20" s="5" t="n">
         <v>0</v>
       </c>
+      <c r="F20" s="5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1034,6 +1104,9 @@
         <v>0</v>
       </c>
       <c r="E21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1174,20 +1247,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:M30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1285,10 +1360,20 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
+          <t>REPARACIÓN ML</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>VALOR</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
           <t>SIN DEFINIR ML</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>TOTAL $</t>
         </is>
@@ -1333,11 +1418,19 @@
         <v/>
       </c>
       <c r="J8" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A8,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A8,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K8" s="13">
-        <f>C8+E8+G8+I8</f>
+        <f>J8*Tarifas!F2</f>
+        <v/>
+      </c>
+      <c r="L8" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A8,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M8" s="13">
+        <f>C8+E8+G8+I8+K8</f>
         <v/>
       </c>
     </row>
@@ -1380,11 +1473,19 @@
         <v/>
       </c>
       <c r="J9" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A9,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A9,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K9" s="13">
-        <f>C9+E9+G9+I9</f>
+        <f>J9*Tarifas!F3</f>
+        <v/>
+      </c>
+      <c r="L9" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A9,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M9" s="13">
+        <f>C9+E9+G9+I9+K9</f>
         <v/>
       </c>
     </row>
@@ -1427,11 +1528,19 @@
         <v/>
       </c>
       <c r="J10" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A10,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A10,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K10" s="13">
-        <f>C10+E10+G10+I10</f>
+        <f>J10*Tarifas!F4</f>
+        <v/>
+      </c>
+      <c r="L10" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A10,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M10" s="13">
+        <f>C10+E10+G10+I10+K10</f>
         <v/>
       </c>
     </row>
@@ -1474,11 +1583,19 @@
         <v/>
       </c>
       <c r="J11" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A11,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A11,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K11" s="13">
-        <f>C11+E11+G11+I11</f>
+        <f>J11*Tarifas!F5</f>
+        <v/>
+      </c>
+      <c r="L11" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A11,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M11" s="13">
+        <f>C11+E11+G11+I11+K11</f>
         <v/>
       </c>
     </row>
@@ -1521,11 +1638,19 @@
         <v/>
       </c>
       <c r="J12" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A12,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A12,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K12" s="13">
-        <f>C12+E12+G12+I12</f>
+        <f>J12*Tarifas!F6</f>
+        <v/>
+      </c>
+      <c r="L12" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A12,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M12" s="13">
+        <f>C12+E12+G12+I12+K12</f>
         <v/>
       </c>
     </row>
@@ -1568,11 +1693,19 @@
         <v/>
       </c>
       <c r="J13" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A13,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A13,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K13" s="13">
-        <f>C13+E13+G13+I13</f>
+        <f>J13*Tarifas!F7</f>
+        <v/>
+      </c>
+      <c r="L13" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A13,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M13" s="13">
+        <f>C13+E13+G13+I13+K13</f>
         <v/>
       </c>
     </row>
@@ -1615,11 +1748,19 @@
         <v/>
       </c>
       <c r="J14" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A14,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A14,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K14" s="13">
-        <f>C14+E14+G14+I14</f>
+        <f>J14*Tarifas!F8</f>
+        <v/>
+      </c>
+      <c r="L14" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A14,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M14" s="13">
+        <f>C14+E14+G14+I14+K14</f>
         <v/>
       </c>
     </row>
@@ -1662,11 +1803,19 @@
         <v/>
       </c>
       <c r="J15" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A15,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A15,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K15" s="13">
-        <f>C15+E15+G15+I15</f>
+        <f>J15*Tarifas!F9</f>
+        <v/>
+      </c>
+      <c r="L15" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A15,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M15" s="13">
+        <f>C15+E15+G15+I15+K15</f>
         <v/>
       </c>
     </row>
@@ -1709,11 +1858,19 @@
         <v/>
       </c>
       <c r="J16" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A16,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A16,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K16" s="13">
-        <f>C16+E16+G16+I16</f>
+        <f>J16*Tarifas!F10</f>
+        <v/>
+      </c>
+      <c r="L16" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A16,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M16" s="13">
+        <f>C16+E16+G16+I16+K16</f>
         <v/>
       </c>
     </row>
@@ -1756,11 +1913,19 @@
         <v/>
       </c>
       <c r="J17" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A17,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A17,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K17" s="13">
-        <f>C17+E17+G17+I17</f>
+        <f>J17*Tarifas!F11</f>
+        <v/>
+      </c>
+      <c r="L17" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A17,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M17" s="13">
+        <f>C17+E17+G17+I17+K17</f>
         <v/>
       </c>
     </row>
@@ -1803,11 +1968,19 @@
         <v/>
       </c>
       <c r="J18" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A18,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A18,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K18" s="13">
-        <f>C18+E18+G18+I18</f>
+        <f>J18*Tarifas!F12</f>
+        <v/>
+      </c>
+      <c r="L18" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A18,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M18" s="13">
+        <f>C18+E18+G18+I18+K18</f>
         <v/>
       </c>
     </row>
@@ -1850,11 +2023,19 @@
         <v/>
       </c>
       <c r="J19" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A19,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A19,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K19" s="13">
-        <f>C19+E19+G19+I19</f>
+        <f>J19*Tarifas!F13</f>
+        <v/>
+      </c>
+      <c r="L19" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A19,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M19" s="13">
+        <f>C19+E19+G19+I19+K19</f>
         <v/>
       </c>
     </row>
@@ -1897,11 +2078,19 @@
         <v/>
       </c>
       <c r="J20" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A20,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A20,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K20" s="13">
-        <f>C20+E20+G20+I20</f>
+        <f>J20*Tarifas!F14</f>
+        <v/>
+      </c>
+      <c r="L20" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A20,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M20" s="13">
+        <f>C20+E20+G20+I20+K20</f>
         <v/>
       </c>
     </row>
@@ -1944,11 +2133,19 @@
         <v/>
       </c>
       <c r="J21" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A21,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A21,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K21" s="13">
-        <f>C21+E21+G21+I21</f>
+        <f>J21*Tarifas!F15</f>
+        <v/>
+      </c>
+      <c r="L21" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A21,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M21" s="13">
+        <f>C21+E21+G21+I21+K21</f>
         <v/>
       </c>
     </row>
@@ -1991,11 +2188,19 @@
         <v/>
       </c>
       <c r="J22" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A22,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A22,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K22" s="13">
-        <f>C22+E22+G22+I22</f>
+        <f>J22*Tarifas!F16</f>
+        <v/>
+      </c>
+      <c r="L22" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A22,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M22" s="13">
+        <f>C22+E22+G22+I22+K22</f>
         <v/>
       </c>
     </row>
@@ -2038,11 +2243,19 @@
         <v/>
       </c>
       <c r="J23" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A23,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A23,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K23" s="13">
-        <f>C23+E23+G23+I23</f>
+        <f>J23*Tarifas!F17</f>
+        <v/>
+      </c>
+      <c r="L23" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A23,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M23" s="13">
+        <f>C23+E23+G23+I23+K23</f>
         <v/>
       </c>
     </row>
@@ -2085,11 +2298,19 @@
         <v/>
       </c>
       <c r="J24" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A24,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A24,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K24" s="13">
-        <f>C24+E24+G24+I24</f>
+        <f>J24*Tarifas!F18</f>
+        <v/>
+      </c>
+      <c r="L24" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A24,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M24" s="13">
+        <f>C24+E24+G24+I24+K24</f>
         <v/>
       </c>
     </row>
@@ -2132,11 +2353,19 @@
         <v/>
       </c>
       <c r="J25" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A25,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A25,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K25" s="13">
-        <f>C25+E25+G25+I25</f>
+        <f>J25*Tarifas!F19</f>
+        <v/>
+      </c>
+      <c r="L25" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A25,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M25" s="13">
+        <f>C25+E25+G25+I25+K25</f>
         <v/>
       </c>
     </row>
@@ -2179,11 +2408,19 @@
         <v/>
       </c>
       <c r="J26" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A26,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A26,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K26" s="13">
-        <f>C26+E26+G26+I26</f>
+        <f>J26*Tarifas!F20</f>
+        <v/>
+      </c>
+      <c r="L26" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A26,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M26" s="13">
+        <f>C26+E26+G26+I26+K26</f>
         <v/>
       </c>
     </row>
@@ -2226,11 +2463,19 @@
         <v/>
       </c>
       <c r="J27" s="12">
-        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A27,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR")</f>
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A27,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$H:$H,"REPARACION")</f>
         <v/>
       </c>
       <c r="K27" s="13">
-        <f>C27+E27+G27+I27</f>
+        <f>J27*Tarifas!F21</f>
+        <v/>
+      </c>
+      <c r="L27" s="12">
+        <f>SUMIFS(Datos!$L:$L,Datos!$E:$E,$A27,Datos!$I:$I,"&gt;="&amp;$G$3,Datos!$I:$I,"&lt;="&amp;$G$4,Datos!$A:$A,IF($D$4="TODAS","*",$D$4),Datos!$G:$G,"SIN DEFINIR",Datos!$H:$H,"&lt;&gt;REPARACION")</f>
+        <v/>
+      </c>
+      <c r="M27" s="13">
+        <f>C27+E27+G27+I27+K27</f>
         <v/>
       </c>
     </row>
@@ -2280,11 +2525,19 @@
         <f>SUM(K8:K27)</f>
         <v/>
       </c>
+      <c r="L28" s="14">
+        <f>SUM(L8:L27)</f>
+        <v/>
+      </c>
+      <c r="M28" s="15">
+        <f>SUM(M8:M27)</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="16" t="inlineStr">
         <is>
-          <t>SIN DEFINIR = juntas sin taller/campo: no se valorizan hasta corregirlas en la obra.</t>
+          <t>SIN DEFINIR = juntas sin taller/campo: no se valorizan hasta corregirlas en la obra. REPARACIÓN = soldadura de reparación de juntas rechazadas (W5-R1…): tarifa positiva para cobrarla o negativa para descontarla.</t>
         </is>
       </c>
     </row>

</xml_diff>